<commit_message>
Add Visual Sync Upload Trial & accumulated improvements
Features:
- New visual-sync-upload.html: Trial feature for manual visual syncing of XML events
  * Isolated from existing upload flows (single-game, batch, reparse)
  * Supports Gaelic Insights and GIU XML formats
  * Step-by-step workflow: game selection → XML upload → event selection → period selection → video scrubbing → sync calculation → review & save
  * Independent angle/period offsets with comprehensive validation
  * Stores sync metadata in game.meta.visualSync

Improvements:
- admin.html: Added "Visual Sync" link to header navigation
- library.html: Division field enhancements from previous session
- cohesion_bulk_upload_template.xlsx: Added ET column mappings for additional camera angles

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cohesion_bulk_upload_template.xlsx
+++ b/cohesion_bulk_upload_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/barrymcguire/Desktop/Cohesion Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89A04D3E-1A17-8547-AEF7-7609C1F33A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A04185F-B31B-B04B-8B35-0BC0F8BE51A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="31920" windowHeight="20180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1200" windowWidth="31920" windowHeight="20180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bulk Upload Manifest" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="140">
   <si>
     <t>xml_file</t>
   </si>
@@ -148,24 +148,15 @@
     <t>Quarter Final</t>
   </si>
   <si>
-    <t>00:55</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
-    <t>Example row. Replace YouTube URL and colours.</t>
-  </si>
-  <si>
     <t>Donegal</t>
   </si>
   <si>
     <t>Down</t>
   </si>
   <si>
-    <t>Example only.</t>
-  </si>
-  <si>
     <t>Cork</t>
   </si>
   <si>
@@ -271,100 +262,13 @@
     <t>Other</t>
   </si>
   <si>
-    <t>Cavan</t>
-  </si>
-  <si>
-    <t>Round 1</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Rgi2ABlwApw</t>
-  </si>
-  <si>
-    <t>56:51</t>
-  </si>
-  <si>
     <t>#ed3327</t>
   </si>
   <si>
-    <t>#171796</t>
-  </si>
-  <si>
-    <t>00:13</t>
-  </si>
-  <si>
-    <t>39:36</t>
-  </si>
-  <si>
     <t>WIDE</t>
   </si>
   <si>
-    <t>https://youtu.be/UM89y1BN1ag</t>
-  </si>
-  <si>
-    <t>Offaly</t>
-  </si>
-  <si>
-    <t>Round 2</t>
-  </si>
-  <si>
-    <t>Round 3</t>
-  </si>
-  <si>
-    <t>https://youtu.be/ZibxPmAmIGs</t>
-  </si>
-  <si>
-    <t>00:32</t>
-  </si>
-  <si>
-    <t>37:10</t>
-  </si>
-  <si>
-    <t>#ffb700</t>
-  </si>
-  <si>
-    <t>https://youtu.be/g1tW1TN7ZSE</t>
-  </si>
-  <si>
-    <t>00:03</t>
-  </si>
-  <si>
-    <t>35:26</t>
-  </si>
-  <si>
-    <t>https://youtu.be/UxrcZ3N0pKc</t>
-  </si>
-  <si>
-    <t>#dd1105</t>
-  </si>
-  <si>
     <t>#ffffff</t>
-  </si>
-  <si>
-    <t>Louth</t>
-  </si>
-  <si>
-    <t>00:27</t>
-  </si>
-  <si>
-    <t>53:23</t>
-  </si>
-  <si>
-    <t>cork-cavan-2026-d2r1.xml</t>
-  </si>
-  <si>
-    <t>louth-cork-2026-d2r2.xml</t>
-  </si>
-  <si>
-    <t>cork-cavan-2026-d2r1</t>
-  </si>
-  <si>
-    <t>louth-cork-2026-d2r2</t>
-  </si>
-  <si>
-    <t>offaly-cork-2026-d2r3.xml</t>
-  </si>
-  <si>
-    <t>offaly-cork-2026-d2r3</t>
   </si>
   <si>
     <t>title</t>
@@ -687,7 +591,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="BulkUploadManifest" displayName="BulkUploadManifest" ref="A1:AH50">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="BulkUploadManifest" displayName="BulkUploadManifest" ref="A1:AH47">
   <tableColumns count="34">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="xml_file"/>
     <tableColumn id="34" xr3:uid="{9933E259-629A-7B42-BF51-43123E21912E}" name="title" dataDxfId="0">
@@ -879,7 +783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH50"/>
+  <dimension ref="A1:AH47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="2" width="37.33203125" customWidth="1"/>
@@ -911,7 +815,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>110</v>
+        <v>78</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>1</v>
@@ -1012,66 +916,67 @@
     </row>
     <row r="2" spans="1:34" ht="25.5" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B2" t="str">
-        <f t="shared" ref="B2:B33" si="0">CONCATENATE(C2, " v ", D2)</f>
-        <v>Cork v Cavan</v>
+        <v>81</v>
+      </c>
+      <c r="B2" s="3" t="str">
+        <f t="shared" ref="B2:B30" si="0">CONCATENATE(C2, " v ", D2)</f>
+        <v>Cork v Meath</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="4">
-        <v>46047</v>
+        <v>46075</v>
       </c>
       <c r="F2" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="H2" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="I2" t="s">
         <v>80</v>
       </c>
+      <c r="I2" s="3" t="s">
+        <v>83</v>
+      </c>
       <c r="J2" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="O2" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="K2" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>38</v>
       </c>
       <c r="P2" s="5"/>
       <c r="Q2" s="5"/>
       <c r="R2" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S2" t="s">
+        <v>76</v>
+      </c>
+      <c r="S2" s="5" t="s">
         <v>87</v>
       </c>
       <c r="T2" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="V2" s="5"/>
+      <c r="W2" s="5"/>
       <c r="X2" s="5"/>
       <c r="Y2" s="5"/>
       <c r="Z2" s="5"/>
@@ -1082,63 +987,69 @@
       <c r="AE2" s="5"/>
       <c r="AF2" s="5"/>
       <c r="AG2" s="5"/>
-      <c r="AH2" s="3" t="s">
-        <v>39</v>
-      </c>
+      <c r="AH2" s="3"/>
     </row>
     <row r="3" spans="1:34" ht="25.5" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="B3" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>Louth v Cork</v>
+        <v>Derry v Cork</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E3" s="4">
-        <v>46054</v>
+        <v>46082</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="H3" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
+      <c r="R3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="S3" t="s">
+        <v>98</v>
+      </c>
+      <c r="T3" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="V3" s="5"/>
       <c r="W3" s="5"/>
       <c r="X3" s="5"/>
@@ -1151,70 +1062,68 @@
       <c r="AE3" s="5"/>
       <c r="AF3" s="5"/>
       <c r="AG3" s="5"/>
-      <c r="AH3" s="3" t="s">
-        <v>42</v>
-      </c>
+      <c r="AH3" s="3"/>
     </row>
     <row r="4" spans="1:34" ht="25.5" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B4" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>Offaly v Cork</v>
+        <v>Cork v Kildare</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>88</v>
+        <v>40</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>43</v>
+        <v>100</v>
       </c>
       <c r="E4" s="4">
-        <v>46068</v>
+        <v>46095</v>
       </c>
       <c r="F4" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="H4" s="3" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P4" s="5"/>
       <c r="Q4" s="5"/>
       <c r="R4" s="5" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="V4" s="5"/>
       <c r="W4" s="5"/>
@@ -1228,70 +1137,68 @@
       <c r="AE4" s="5"/>
       <c r="AF4" s="5"/>
       <c r="AG4" s="5"/>
-      <c r="AH4" s="3" t="s">
-        <v>42</v>
-      </c>
+      <c r="AH4" s="3"/>
     </row>
     <row r="5" spans="1:34" ht="25.5" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>113</v>
+        <v>138</v>
       </c>
       <c r="B5" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>Cork v Meath</v>
+        <v>Tyrone v Cork</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>43</v>
+        <v>113</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="4">
+        <v>46103</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="H5" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E5" s="4">
-        <v>46075</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>116</v>
-      </c>
       <c r="K5" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>118</v>
+        <v>75</v>
       </c>
       <c r="N5" s="3" t="s">
-        <v>114</v>
+        <v>139</v>
       </c>
       <c r="O5" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P5" s="5"/>
       <c r="Q5" s="5"/>
       <c r="R5" s="5" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="V5" s="5"/>
       <c r="W5" s="5"/>
@@ -1309,64 +1216,62 @@
     </row>
     <row r="6" spans="1:34" ht="25.5" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B6" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>Derry v Cork</v>
+        <v>Donegal v Down</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>124</v>
+        <v>38</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E6" s="4">
-        <v>46082</v>
+        <v>46138</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>71</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="G6" s="3"/>
       <c r="H6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="N6" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="K6" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="L6" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="M6" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="N6" s="3" t="s">
-        <v>126</v>
-      </c>
       <c r="O6" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P6" s="5"/>
       <c r="Q6" s="5"/>
       <c r="R6" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S6" t="s">
-        <v>130</v>
+        <v>76</v>
+      </c>
+      <c r="S6" s="5" t="s">
+        <v>125</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="V6" s="5"/>
       <c r="W6" s="5"/>
@@ -1384,64 +1289,62 @@
     </row>
     <row r="7" spans="1:34" ht="25.5" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B7" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>Cork v Kildare</v>
+        <v>Fermanagh v Armagh</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="4">
+        <v>46137</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="M7" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="E7" s="4">
-        <v>46095</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>100</v>
-      </c>
       <c r="N7" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="O7" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P7" s="5"/>
       <c r="Q7" s="5"/>
       <c r="R7" s="5" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="T7" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="V7" s="5"/>
       <c r="W7" s="5"/>
@@ -1458,66 +1361,30 @@
       <c r="AH7" s="3"/>
     </row>
     <row r="8" spans="1:34" ht="25.5" customHeight="1">
-      <c r="A8" s="3" t="s">
-        <v>170</v>
-      </c>
+      <c r="A8" s="3"/>
       <c r="B8" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>Tyrone v Cork</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E8" s="4">
-        <v>46103</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>38</v>
-      </c>
+        <v xml:space="preserve"> v </v>
+      </c>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="4"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
       <c r="P8" s="5"/>
       <c r="Q8" s="5"/>
-      <c r="R8" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S8" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="T8" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="U8" s="5" t="s">
-        <v>149</v>
-      </c>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
       <c r="V8" s="5"/>
       <c r="W8" s="5"/>
       <c r="X8" s="5"/>
@@ -1533,64 +1400,30 @@
       <c r="AH8" s="3"/>
     </row>
     <row r="9" spans="1:34" ht="25.5" customHeight="1">
-      <c r="A9" s="3" t="s">
-        <v>156</v>
-      </c>
+      <c r="A9" s="3"/>
       <c r="B9" s="3" t="str">
-        <f>CONCATENATE(C9, " v ", D9)</f>
-        <v>Donegal v Down</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E9" s="4">
-        <v>46138</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>35</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="3"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="L9" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="M9" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="N9" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>38</v>
-      </c>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
       <c r="P9" s="5"/>
       <c r="Q9" s="5"/>
-      <c r="R9" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S9" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="T9" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="U9" s="5" t="s">
-        <v>158</v>
-      </c>
+      <c r="R9" s="5"/>
+      <c r="S9" s="5"/>
+      <c r="T9" s="5"/>
+      <c r="U9" s="5"/>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
       <c r="X9" s="5"/>
@@ -1606,64 +1439,30 @@
       <c r="AH9" s="3"/>
     </row>
     <row r="10" spans="1:34" ht="25.5" customHeight="1">
-      <c r="A10" s="3" t="s">
-        <v>162</v>
-      </c>
+      <c r="A10" s="3"/>
       <c r="B10" s="3" t="str">
-        <f>CONCATENATE(C10, " v ", D10)</f>
-        <v>Fermanagh v Armagh</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="4">
-        <v>46137</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>35</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="4"/>
+      <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>166</v>
-      </c>
-      <c r="K10" s="5" t="s">
-        <v>165</v>
-      </c>
-      <c r="L10" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>38</v>
-      </c>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
       <c r="P10" s="5"/>
       <c r="Q10" s="5"/>
-      <c r="R10" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="S10" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="T10" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="U10" s="5" t="s">
-        <v>169</v>
-      </c>
+      <c r="R10" s="5"/>
+      <c r="S10" s="5"/>
+      <c r="T10" s="5"/>
+      <c r="U10" s="5"/>
       <c r="V10" s="5"/>
       <c r="W10" s="5"/>
       <c r="X10" s="5"/>
@@ -1680,7 +1479,10 @@
     </row>
     <row r="11" spans="1:34" ht="25.5" customHeight="1">
       <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
+      <c r="B11" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="4"/>
@@ -1716,7 +1518,10 @@
     </row>
     <row r="12" spans="1:34" ht="25.5" customHeight="1">
       <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
+      <c r="B12" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
       <c r="E12" s="4"/>
@@ -1752,7 +1557,10 @@
     </row>
     <row r="13" spans="1:34" ht="25.5" customHeight="1">
       <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
+      <c r="B13" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="4"/>
@@ -1788,7 +1596,10 @@
     </row>
     <row r="14" spans="1:34" ht="25.5" customHeight="1">
       <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
+      <c r="B14" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
       <c r="E14" s="4"/>
@@ -1824,7 +1635,10 @@
     </row>
     <row r="15" spans="1:34" ht="25.5" customHeight="1">
       <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
+      <c r="B15" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
       <c r="E15" s="4"/>
@@ -1860,7 +1674,10 @@
     </row>
     <row r="16" spans="1:34" ht="25.5" customHeight="1">
       <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
+      <c r="B16" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
       <c r="E16" s="4"/>
@@ -1896,7 +1713,10 @@
     </row>
     <row r="17" spans="1:34" ht="25.5" customHeight="1">
       <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
+      <c r="B17" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
       <c r="E17" s="4"/>
@@ -1932,7 +1752,10 @@
     </row>
     <row r="18" spans="1:34" ht="25.5" customHeight="1">
       <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
+      <c r="B18" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
       <c r="E18" s="4"/>
@@ -1968,7 +1791,10 @@
     </row>
     <row r="19" spans="1:34" ht="25.5" customHeight="1">
       <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
+      <c r="B19" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
       <c r="E19" s="4"/>
@@ -2004,7 +1830,10 @@
     </row>
     <row r="20" spans="1:34" ht="25.5" customHeight="1">
       <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
+      <c r="B20" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
       <c r="E20" s="4"/>
@@ -2040,7 +1869,10 @@
     </row>
     <row r="21" spans="1:34" ht="25.5" customHeight="1">
       <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
+      <c r="B21" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="4"/>
@@ -2076,7 +1908,10 @@
     </row>
     <row r="22" spans="1:34" ht="25.5" customHeight="1">
       <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
+      <c r="B22" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
       <c r="E22" s="4"/>
@@ -2112,7 +1947,10 @@
     </row>
     <row r="23" spans="1:34" ht="25.5" customHeight="1">
       <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
+      <c r="B23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
       <c r="E23" s="4"/>
@@ -2148,7 +1986,10 @@
     </row>
     <row r="24" spans="1:34" ht="25.5" customHeight="1">
       <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
+      <c r="B24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
       <c r="E24" s="4"/>
@@ -2184,7 +2025,10 @@
     </row>
     <row r="25" spans="1:34" ht="25.5" customHeight="1">
       <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
+      <c r="B25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
       <c r="E25" s="4"/>
@@ -2220,7 +2064,10 @@
     </row>
     <row r="26" spans="1:34" ht="25.5" customHeight="1">
       <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
+      <c r="B26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="4"/>
@@ -2256,7 +2103,10 @@
     </row>
     <row r="27" spans="1:34" ht="25.5" customHeight="1">
       <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
+      <c r="B27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
       <c r="E27" s="4"/>
@@ -2292,7 +2142,10 @@
     </row>
     <row r="28" spans="1:34" ht="25.5" customHeight="1">
       <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
+      <c r="B28" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
       <c r="E28" s="4"/>
@@ -2328,7 +2181,10 @@
     </row>
     <row r="29" spans="1:34" ht="25.5" customHeight="1">
       <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
+      <c r="B29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
       <c r="E29" s="4"/>
@@ -2364,7 +2220,10 @@
     </row>
     <row r="30" spans="1:34" ht="25.5" customHeight="1">
       <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
+      <c r="B30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
       <c r="E30" s="4"/>
@@ -2400,7 +2259,10 @@
     </row>
     <row r="31" spans="1:34" ht="25.5" customHeight="1">
       <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
+      <c r="B31" s="3" t="str">
+        <f t="shared" ref="B31:B62" si="1">CONCATENATE(C31, " v ", D31)</f>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
       <c r="E31" s="4"/>
@@ -2436,7 +2298,10 @@
     </row>
     <row r="32" spans="1:34" ht="25.5" customHeight="1">
       <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
+      <c r="B32" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
       <c r="E32" s="4"/>
@@ -2472,7 +2337,10 @@
     </row>
     <row r="33" spans="1:34" ht="25.5" customHeight="1">
       <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
+      <c r="B33" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
       <c r="E33" s="4"/>
@@ -2508,7 +2376,10 @@
     </row>
     <row r="34" spans="1:34" ht="25.5" customHeight="1">
       <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
+      <c r="B34" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
       <c r="E34" s="4"/>
@@ -2544,7 +2415,10 @@
     </row>
     <row r="35" spans="1:34" ht="25.5" customHeight="1">
       <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
+      <c r="B35" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
       <c r="E35" s="4"/>
@@ -2580,7 +2454,10 @@
     </row>
     <row r="36" spans="1:34" ht="25.5" customHeight="1">
       <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
+      <c r="B36" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
       <c r="E36" s="4"/>
@@ -2616,7 +2493,10 @@
     </row>
     <row r="37" spans="1:34" ht="25.5" customHeight="1">
       <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
+      <c r="B37" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
       <c r="E37" s="4"/>
@@ -2652,7 +2532,10 @@
     </row>
     <row r="38" spans="1:34" ht="25.5" customHeight="1">
       <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
+      <c r="B38" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
       <c r="E38" s="4"/>
@@ -2688,7 +2571,10 @@
     </row>
     <row r="39" spans="1:34" ht="25.5" customHeight="1">
       <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
+      <c r="B39" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="4"/>
@@ -2724,7 +2610,10 @@
     </row>
     <row r="40" spans="1:34" ht="25.5" customHeight="1">
       <c r="A40" s="3"/>
-      <c r="B40" s="3"/>
+      <c r="B40" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
       <c r="E40" s="4"/>
@@ -2760,7 +2649,10 @@
     </row>
     <row r="41" spans="1:34" ht="25.5" customHeight="1">
       <c r="A41" s="3"/>
-      <c r="B41" s="3"/>
+      <c r="B41" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
       <c r="E41" s="4"/>
@@ -2796,7 +2688,10 @@
     </row>
     <row r="42" spans="1:34" ht="25.5" customHeight="1">
       <c r="A42" s="3"/>
-      <c r="B42" s="3"/>
+      <c r="B42" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
       <c r="E42" s="4"/>
@@ -2832,7 +2727,10 @@
     </row>
     <row r="43" spans="1:34" ht="25.5" customHeight="1">
       <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
+      <c r="B43" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C43" s="3"/>
       <c r="D43" s="3"/>
       <c r="E43" s="4"/>
@@ -2868,7 +2766,10 @@
     </row>
     <row r="44" spans="1:34" ht="25.5" customHeight="1">
       <c r="A44" s="3"/>
-      <c r="B44" s="3"/>
+      <c r="B44" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C44" s="3"/>
       <c r="D44" s="3"/>
       <c r="E44" s="4"/>
@@ -2904,7 +2805,10 @@
     </row>
     <row r="45" spans="1:34" ht="25.5" customHeight="1">
       <c r="A45" s="3"/>
-      <c r="B45" s="3"/>
+      <c r="B45" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C45" s="3"/>
       <c r="D45" s="3"/>
       <c r="E45" s="4"/>
@@ -2940,7 +2844,10 @@
     </row>
     <row r="46" spans="1:34" ht="25.5" customHeight="1">
       <c r="A46" s="3"/>
-      <c r="B46" s="3"/>
+      <c r="B46" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C46" s="3"/>
       <c r="D46" s="3"/>
       <c r="E46" s="4"/>
@@ -2976,7 +2883,10 @@
     </row>
     <row r="47" spans="1:34" ht="25.5" customHeight="1">
       <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
+      <c r="B47" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v xml:space="preserve"> v </v>
+      </c>
       <c r="C47" s="3"/>
       <c r="D47" s="3"/>
       <c r="E47" s="4"/>
@@ -3010,114 +2920,6 @@
       <c r="AG47" s="5"/>
       <c r="AH47" s="3"/>
     </row>
-    <row r="48" spans="1:34" ht="25.5" customHeight="1">
-      <c r="A48" s="3"/>
-      <c r="B48" s="3"/>
-      <c r="C48" s="3"/>
-      <c r="D48" s="3"/>
-      <c r="E48" s="4"/>
-      <c r="F48" s="3"/>
-      <c r="G48" s="3"/>
-      <c r="H48" s="3"/>
-      <c r="I48" s="3"/>
-      <c r="J48" s="5"/>
-      <c r="K48" s="5"/>
-      <c r="L48" s="5"/>
-      <c r="M48" s="5"/>
-      <c r="N48" s="3"/>
-      <c r="O48" s="3"/>
-      <c r="P48" s="5"/>
-      <c r="Q48" s="5"/>
-      <c r="R48" s="5"/>
-      <c r="S48" s="5"/>
-      <c r="T48" s="5"/>
-      <c r="U48" s="5"/>
-      <c r="V48" s="5"/>
-      <c r="W48" s="5"/>
-      <c r="X48" s="5"/>
-      <c r="Y48" s="5"/>
-      <c r="Z48" s="5"/>
-      <c r="AA48" s="5"/>
-      <c r="AB48" s="5"/>
-      <c r="AC48" s="5"/>
-      <c r="AD48" s="5"/>
-      <c r="AE48" s="5"/>
-      <c r="AF48" s="5"/>
-      <c r="AG48" s="5"/>
-      <c r="AH48" s="3"/>
-    </row>
-    <row r="49" spans="1:34" ht="25.5" customHeight="1">
-      <c r="A49" s="3"/>
-      <c r="B49" s="3"/>
-      <c r="C49" s="3"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="4"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-      <c r="J49" s="5"/>
-      <c r="K49" s="5"/>
-      <c r="L49" s="5"/>
-      <c r="M49" s="5"/>
-      <c r="N49" s="3"/>
-      <c r="O49" s="3"/>
-      <c r="P49" s="5"/>
-      <c r="Q49" s="5"/>
-      <c r="R49" s="5"/>
-      <c r="S49" s="5"/>
-      <c r="T49" s="5"/>
-      <c r="U49" s="5"/>
-      <c r="V49" s="5"/>
-      <c r="W49" s="5"/>
-      <c r="X49" s="5"/>
-      <c r="Y49" s="5"/>
-      <c r="Z49" s="5"/>
-      <c r="AA49" s="5"/>
-      <c r="AB49" s="5"/>
-      <c r="AC49" s="5"/>
-      <c r="AD49" s="5"/>
-      <c r="AE49" s="5"/>
-      <c r="AF49" s="5"/>
-      <c r="AG49" s="5"/>
-      <c r="AH49" s="3"/>
-    </row>
-    <row r="50" spans="1:34" ht="25.5" customHeight="1">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="3"/>
-      <c r="D50" s="3"/>
-      <c r="E50" s="4"/>
-      <c r="F50" s="3"/>
-      <c r="G50" s="3"/>
-      <c r="H50" s="3"/>
-      <c r="I50" s="3"/>
-      <c r="J50" s="5"/>
-      <c r="K50" s="5"/>
-      <c r="L50" s="5"/>
-      <c r="M50" s="5"/>
-      <c r="N50" s="3"/>
-      <c r="O50" s="3"/>
-      <c r="P50" s="5"/>
-      <c r="Q50" s="5"/>
-      <c r="R50" s="5"/>
-      <c r="S50" s="5"/>
-      <c r="T50" s="5"/>
-      <c r="U50" s="5"/>
-      <c r="V50" s="5"/>
-      <c r="W50" s="5"/>
-      <c r="X50" s="5"/>
-      <c r="Y50" s="5"/>
-      <c r="Z50" s="5"/>
-      <c r="AA50" s="5"/>
-      <c r="AB50" s="5"/>
-      <c r="AC50" s="5"/>
-      <c r="AD50" s="5"/>
-      <c r="AE50" s="5"/>
-      <c r="AF50" s="5"/>
-      <c r="AG50" s="5"/>
-      <c r="AH50" s="3"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -3130,19 +2932,19 @@
           <x14:formula1>
             <xm:f>Lists!$A$2:$A$8</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F50</xm:sqref>
+          <xm:sqref>F8:F47 F2:F7</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Lists!$E$2:$E$6</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G50</xm:sqref>
+          <xm:sqref>G8:G47 G2:G7</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Lists!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>O2:O50</xm:sqref>
+          <xm:sqref>O8:O47 O2:O7</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3161,7 +2963,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15">
       <c r="A1" s="9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="11"/>
@@ -3173,50 +2975,50 @@
     </row>
     <row r="3" spans="1:8" ht="31">
       <c r="A3" s="6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="31">
       <c r="A4" s="6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="16">
       <c r="A5" s="6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="31">
       <c r="A6" s="6" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="16">
       <c r="A7" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="16">
       <c r="A8" s="6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="16">
@@ -3224,31 +3026,31 @@
         <v>12</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="16">
       <c r="A10" s="6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="31">
       <c r="A11" s="6" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="16">
       <c r="A12" s="6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -3269,26 +3071,26 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -3296,41 +3098,41 @@
         <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E5" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>